<commit_message>
Updated login and request access page
</commit_message>
<xml_diff>
--- a/Access.xlsx
+++ b/Access.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varshnem\Python Training\IB Cricket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44ED4CF-8C9C-4960-AF65-3015E5E1A059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F7A618-E904-46C4-A63C-2176CDABF3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28692" yWindow="-108" windowWidth="51816" windowHeight="21096" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>Username</t>
   </si>
@@ -47,10 +47,37 @@
     <t>Approved</t>
   </si>
   <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>Scorekeeper</t>
+  </si>
+  <si>
+    <t>Viewer</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
     <t>RequestedOn</t>
+  </si>
+  <si>
+    <t>sss</t>
+  </si>
+  <si>
+    <t>ssdfgfg</t>
+  </si>
+  <si>
+    <t>2026-07-23 22:30</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>2026-07-23 23:06</t>
+  </si>
+  <si>
+    <t>admin</t>
   </si>
 </sst>
 </file>
@@ -430,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="15" customWidth="1"/>
@@ -465,10 +492,32 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -477,24 +526,49 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="5" width="21.5546875" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial commit - Season 2 and Season 3 Dashboard
</commit_message>
<xml_diff>
--- a/Access.xlsx
+++ b/Access.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varshnem\Python Training\IB Cricket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F7A618-E904-46C4-A63C-2176CDABF3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0310F122-42F9-49A4-A8A5-3F532DE37B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>Username</t>
   </si>
@@ -35,24 +35,21 @@
     <t>Status</t>
   </si>
   <si>
-    <t>manish</t>
-  </si>
-  <si>
-    <t>admin123</t>
-  </si>
-  <si>
     <t>Admin</t>
   </si>
   <si>
     <t>Approved</t>
   </si>
   <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>Scorekeeper</t>
+  </si>
+  <si>
     <t>user</t>
   </si>
   <si>
-    <t>Scorekeeper</t>
-  </si>
-  <si>
     <t>Viewer</t>
   </si>
   <si>
@@ -62,22 +59,13 @@
     <t>RequestedOn</t>
   </si>
   <si>
-    <t>sss</t>
-  </si>
-  <si>
-    <t>ssdfgfg</t>
-  </si>
-  <si>
-    <t>2026-07-23 22:30</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>2026-07-23 23:06</t>
-  </si>
-  <si>
-    <t>admin</t>
+    <t>admin123*</t>
+  </si>
+  <si>
+    <t>scorekeeper</t>
+  </si>
+  <si>
+    <t>scorekeeper123*</t>
   </si>
 </sst>
 </file>
@@ -460,7 +448,9 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="15" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -479,30 +469,30 @@
     </row>
     <row r="2" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -513,10 +503,10 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -526,49 +516,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="14.44140625" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="4" max="5" width="14.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
         <v>11</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move cricket app to Google Sheets
</commit_message>
<xml_diff>
--- a/Access.xlsx
+++ b/Access.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varshnem\Python Training\IB Cricket\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0310F122-42F9-49A4-A8A5-3F532DE37B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01432A30-BFDB-4FDF-803C-50D0444F3ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -467,7 +467,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="17.399999999999999" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>

</xml_diff>